<commit_message>
Add create_index_sheet function with clickable links
- New create_index_sheet() function creates table of contents
- Automatically generates links to all data sheets
- Each data sheet has 'Back to Index' link
- Index sheet appears last (openxlsx2 limitation)
- German formatting and styling maintained
- Demo shows complete multi-sheet workflow
</commit_message>
<xml_diff>
--- a/projects/r-export-excel/output/demo_statistik_mehrere_sheets.xlsx
+++ b/projects/r-export-excel/output/demo_statistik_mehrere_sheets.xlsx
@@ -1144,10 +1144,10 @@
   <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="30.711"/>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="40.711"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row customHeight="1" ht="30" r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Inhaltsverzeichnis</t>

</xml_diff>

<commit_message>
Implement two-step index creation for correct sheet ordering
- Add init_index_sheet() to create placeholder as first sheet
- Add update_index_sheet() to populate with links after data sheets added
- Keep create_index_sheet() as legacy convenience function
- Index now correctly appears as FIRST sheet in workbook
- Demo updated to show proper workflow: init → add data → update
- Sheet order: Index, Bevölkerung, Wirtschaft, Bildung
</commit_message>
<xml_diff>
--- a/projects/r-export-excel/output/demo_statistik_mehrere_sheets.xlsx
+++ b/projects/r-export-excel/output/demo_statistik_mehrere_sheets.xlsx
@@ -6,10 +6,10 @@
     <workbookView activeTab="0" firstSheet="0" windowHeight="13125" windowWidth="13125" xWindow="0" yWindow="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Bevölkerung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Wirtschaft" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Bildung" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Index" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bevölkerung" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Wirtschaft" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bildung" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -417,6 +417,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="40.711"/>
+  </cols>
+  <sheetData>
+    <row customHeight="1" ht="30" r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Inhaltsverzeichnis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="str">
+        <f>HYPERLINK("#Bevölkerung!A1", "Bevölkerung")</f>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="str">
+        <f>HYPERLINK("#Wirtschaft!A1", "Wirtschaft")</f>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="str">
+        <f>HYPERLINK("#Bildung!A1", "Bildung")</f>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -688,7 +725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -910,7 +947,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1137,41 +1174,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="40.711"/>
-  </cols>
-  <sheetData>
-    <row customHeight="1" ht="30" r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Inhaltsverzeichnis</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="str">
-        <f>HYPERLINK("#Bevölkerung!A1", "Bevölkerung")</f>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="str">
-        <f>HYPERLINK("#Wirtschaft!A1", "Wirtschaft")</f>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="str">
-        <f>HYPERLINK("#Bildung!A1", "Bildung")</f>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions gridLines="1" gridLinesSet="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix number formatting, link colors, and header backgrounds
- Use add_numfmt() to apply German number format (# ### ##0,00) to all data cells
- Use add_font() with underline='single' for blue hyperlink styling
- Use add_fill() to explicitly apply light grey background to headers
- Replace create_cell_style() approach with direct formatting functions
- Fixes display of hundreds separator (space), comma decimals
- Fixes blue link color (0563C1) for all hyperlinks
- Fixes light grey header background (D9D9D9)
</commit_message>
<xml_diff>
--- a/projects/r-export-excel/output/demo_statistik_mehrere_sheets.xlsx
+++ b/projects/r-export-excel/output/demo_statistik_mehrere_sheets.xlsx
@@ -16,7 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1">
+  <numFmts count="3">
+    <numFmt numFmtId="165" formatCode="# ### ##0,00"/>
+    <numFmt numFmtId="166" formatCode="# ### ##0,00"/>
+    <numFmt numFmtId="167" formatCode="# ### ##0,00"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -24,13 +29,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <color rgb="FF0563C1"/>
+      <name val="Aptos Narrow"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -45,9 +61,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0"/>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyFill="1" borderId="0" fillId="2" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="165" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="166" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="167" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,7 +445,7 @@
   </cols>
   <sheetData>
     <row customHeight="1" ht="30" r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Inhaltsverzeichnis</t>
         </is>
@@ -471,242 +492,242 @@
       </c>
     </row>
     <row customHeight="1" ht="25" r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bevölkerungsstatistik nach Bundesländern</t>
         </is>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Verwaltung</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Bevölkerung</t>
         </is>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Geographie</t>
         </is>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Bundesland</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Einwohner_Gesamt</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Einwohner_Maennlich</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Einwohner_Weiblich</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Flaeche_km2</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Dichte_pro_km2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Baden-Württemberg</t>
         </is>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="4">
         <v>11280257</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="4">
         <v>5589321</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="4">
         <v>5690936</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="4">
         <v>35748</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="4">
         <v>315.5</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Bayern</t>
         </is>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="4">
         <v>13369393</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="4">
         <v>6631044</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="4">
         <v>6738349</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="4">
         <v>70541</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="4">
         <v>189.5</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Berlin</t>
         </is>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="4">
         <v>3769495</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="4">
         <v>1864218</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="4">
         <v>1905277</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="4">
         <v>892</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="4">
         <v>4227.1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Brandenburg</t>
         </is>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="4">
         <v>2573138</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="4">
         <v>1283629</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="4">
         <v>1289509</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="4">
         <v>29654</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="4">
         <v>86.8</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Bremen</t>
         </is>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="4">
         <v>676463</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="4">
         <v>333912</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="4">
         <v>342551</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="4">
         <v>420</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="4">
         <v>1610.6</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Hamburg</t>
         </is>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="4">
         <v>1906411</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="4">
         <v>950287</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="4">
         <v>956124</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="4">
         <v>755</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="4">
         <v>2525.3</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Hessen</t>
         </is>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="4">
         <v>6391360</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="4">
         <v>3168234</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="4">
         <v>3223126</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="4">
         <v>21116</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="4">
         <v>302.6</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Niedersachsen</t>
         </is>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="4">
         <v>8140242</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="4">
         <v>4042628</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="4">
         <v>4097614</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="4">
         <v>47710</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="4">
         <v>170.6</v>
       </c>
     </row>
@@ -746,188 +767,188 @@
       </c>
     </row>
     <row customHeight="1" ht="25" r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Wirtschaftsindikatoren Deutschland</t>
         </is>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Zeitraum</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Bruttoinlandsprodukt (Mrd. €)</t>
         </is>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Arbeitsmarkt</t>
         </is>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="F3" s="3"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Inflation (%)</t>
         </is>
       </c>
-      <c r="H3" s="1"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Jahr</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>BIP_Nominal</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>BIP_Real</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>BIP_Wachstum</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Arbeitslose</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Arbeitslosenquote</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Inflation</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Inflation_Energie</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1">
+      <c r="A5" s="5">
         <v>2020</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="5">
         <v>3332</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="5">
         <v>3280.5</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="5">
         <v>-3.8</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="5">
         <v>2695000</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="5">
         <v>5.9</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="5">
         <v>0.5</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="5">
         <v>-5.2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1">
+      <c r="A6" s="5">
         <v>2021</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="5">
         <v>3617.5</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="5">
         <v>3385.1</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="5">
         <v>3.2</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="5">
         <v>2613000</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="5">
         <v>5.7</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="5">
         <v>3.1</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="5">
         <v>4.5</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1">
+      <c r="A7" s="5">
         <v>2022</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="5">
         <v>3876.8</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="5">
         <v>3445.8</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="5">
         <v>1.8</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="5">
         <v>2418000</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="5">
         <v>5.3</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="5">
         <v>6.9</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="5">
         <v>34.7</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1">
+      <c r="A8" s="5">
         <v>2023</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="5">
         <v>4121.2</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="5">
         <v>3435.5</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="5">
         <v>-0.3</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="5">
         <v>2607000</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="5">
         <v>5.7</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="5">
         <v>5.9</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="5">
         <v>-2.7</v>
       </c>
     </row>
@@ -966,198 +987,198 @@
       </c>
     </row>
     <row customHeight="1" ht="25" r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bildungsausgaben nach Bereichen</t>
         </is>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Bereich</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Ausgaben (Mio. €)</t>
         </is>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Personen</t>
         </is>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Bildungsbereich</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Personal_Mio</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Sachmittel_Mio</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Investitionen_Mio</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Schueler</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Lehrer</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Kindergärten</t>
         </is>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="6">
         <v>4521.3</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="6">
         <v>2134.7</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="6">
         <v>1794.5</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="6">
         <v>745200</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="6">
         <v>52340</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Grundschulen</t>
         </is>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="6">
         <v>8234.5</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="6">
         <v>4123.8</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="6">
         <v>2872.5</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="6">
         <v>2834500</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="6">
         <v>198230</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Weiterführende Schulen</t>
         </is>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="6">
         <v>12456.8</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="6">
         <v>6234.1</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="6">
         <v>3876.4</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="6">
         <v>8456300</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="6">
         <v>534200</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Berufsschulen</t>
         </is>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="6">
         <v>3124.6</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="6">
         <v>1678.9</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="6">
         <v>1088.6</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="6">
         <v>2567800</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="6">
         <v>89450</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Hochschulen</t>
         </is>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="6">
         <v>18234.2</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="6">
         <v>9123.4</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="6">
         <v>4793.3</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="6">
         <v>2948600</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="6">
         <v>412300</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Erwachsenenbildung</t>
         </is>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="6">
         <v>1245.8</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="6">
         <v>678.3</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="6">
         <v>416.6</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="6">
         <v>156700</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="6">
         <v>12450</v>
       </c>
     </row>

</xml_diff>